<commit_message>
Atualiza dados do estoque e compras
</commit_message>
<xml_diff>
--- a/data-source/COMPRABASES.xlsx
+++ b/data-source/COMPRABASES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/Relatórios SMART-STOCK/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/SMART-STOCK/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{4387A5D2-32EA-4489-B23A-44C699D43E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A22DD465-1E58-4CF6-A523-141C0DD17208}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{4387A5D2-32EA-4489-B23A-44C699D43E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6444C48-3030-4A02-9062-CB80BBD9884B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,10 +193,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[Blue]###########0;[Red]\-###########0"/>
     <numFmt numFmtId="165" formatCode="[Blue]###,###,###,##0.000;[Red]\-###,###,###,##0.000"/>
     <numFmt numFmtId="166" formatCode="[Blue]###,###,###,##0.0000;[Red]\-###,###,###,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000_ ;[Red]\-#,##0.000\ "/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -238,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -246,6 +247,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -261,10 +263,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -587,7 +585,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -643,7 +641,7 @@
         <v>46</v>
       </c>
       <c r="F2" s="6">
-        <v>12800</v>
+        <v>15545</v>
       </c>
       <c r="G2" s="3">
         <v>1.23</v>
@@ -1241,7 +1239,7 @@
         <v>46</v>
       </c>
       <c r="F25" s="6">
-        <v>15200</v>
+        <v>17467</v>
       </c>
       <c r="G25" s="3">
         <v>1.23</v>
@@ -1319,7 +1317,7 @@
         <v>46</v>
       </c>
       <c r="F28" s="6">
-        <v>28000</v>
+        <v>30109</v>
       </c>
       <c r="G28" s="3">
         <v>1.23</v>
@@ -1735,7 +1733,7 @@
         <v>46</v>
       </c>
       <c r="F44" s="6">
-        <v>3000</v>
+        <v>5395</v>
       </c>
       <c r="G44" s="3">
         <v>1.75</v>
@@ -1865,7 +1863,7 @@
         <v>46</v>
       </c>
       <c r="F49" s="6">
-        <v>8000</v>
+        <v>9811</v>
       </c>
       <c r="G49" s="3">
         <v>1.75</v>
@@ -2549,6 +2547,18 @@
       <c r="H75" s="5">
         <v>46337</v>
       </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F77" s="6"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F78" s="6"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F79" s="7"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F80" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H75" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Atualiza dashboard e relatórios
</commit_message>
<xml_diff>
--- a/data-source/COMPRABASES.xlsx
+++ b/data-source/COMPRABASES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/SMART-STOCK/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{4387A5D2-32EA-4489-B23A-44C699D43E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6444C48-3030-4A02-9062-CB80BBD9884B}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{4387A5D2-32EA-4489-B23A-44C699D43E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45A81481-E632-48FC-970C-143468D24089}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -667,7 +667,7 @@
         <v>46</v>
       </c>
       <c r="F3" s="6">
-        <v>3600</v>
+        <v>3573</v>
       </c>
       <c r="G3" s="3">
         <v>1.23</v>
@@ -693,7 +693,7 @@
         <v>46</v>
       </c>
       <c r="F4" s="6">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="G4" s="3">
         <v>1.23</v>
@@ -719,7 +719,7 @@
         <v>46</v>
       </c>
       <c r="F5" s="6">
-        <v>1200</v>
+        <v>1212</v>
       </c>
       <c r="G5" s="3">
         <v>1.23</v>
@@ -745,7 +745,7 @@
         <v>46</v>
       </c>
       <c r="F6" s="6">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="G6" s="3">
         <v>1.23</v>
@@ -771,7 +771,7 @@
         <v>46</v>
       </c>
       <c r="F7" s="6">
-        <v>1600</v>
+        <v>1727</v>
       </c>
       <c r="G7" s="3">
         <v>1.23</v>
@@ -797,7 +797,7 @@
         <v>46</v>
       </c>
       <c r="F8" s="6">
-        <v>3400</v>
+        <v>3263</v>
       </c>
       <c r="G8" s="3">
         <v>1.23</v>
@@ -823,7 +823,7 @@
         <v>46</v>
       </c>
       <c r="F9" s="6">
-        <v>3800</v>
+        <v>3870</v>
       </c>
       <c r="G9" s="3">
         <v>1.23</v>
@@ -849,7 +849,7 @@
         <v>46</v>
       </c>
       <c r="F10" s="6">
-        <v>4000</v>
+        <v>3802</v>
       </c>
       <c r="G10" s="3">
         <v>1.23</v>
@@ -875,7 +875,7 @@
         <v>46</v>
       </c>
       <c r="F11" s="6">
-        <v>3200</v>
+        <v>3395</v>
       </c>
       <c r="G11" s="3">
         <v>1.23</v>
@@ -901,7 +901,7 @@
         <v>46</v>
       </c>
       <c r="F12" s="6">
-        <v>3200</v>
+        <v>4054</v>
       </c>
       <c r="G12" s="3">
         <v>1.23</v>
@@ -927,7 +927,7 @@
         <v>46</v>
       </c>
       <c r="F13" s="6">
-        <v>5000</v>
+        <v>6082</v>
       </c>
       <c r="G13" s="3">
         <v>1.23</v>
@@ -953,7 +953,7 @@
         <v>46</v>
       </c>
       <c r="F14" s="6">
-        <v>3600</v>
+        <v>3690</v>
       </c>
       <c r="G14" s="3">
         <v>1.23</v>
@@ -979,7 +979,7 @@
         <v>46</v>
       </c>
       <c r="F15" s="6">
-        <v>1200</v>
+        <v>1260</v>
       </c>
       <c r="G15" s="3">
         <v>1.23</v>
@@ -1005,7 +1005,7 @@
         <v>46</v>
       </c>
       <c r="F16" s="6">
-        <v>800</v>
+        <v>830</v>
       </c>
       <c r="G16" s="3">
         <v>1.23</v>
@@ -1031,7 +1031,7 @@
         <v>46</v>
       </c>
       <c r="F17" s="6">
-        <v>4600</v>
+        <v>4951</v>
       </c>
       <c r="G17" s="3">
         <v>1.23</v>
@@ -1057,7 +1057,7 @@
         <v>46</v>
       </c>
       <c r="F18" s="6">
-        <v>2400</v>
+        <v>2396</v>
       </c>
       <c r="G18" s="3">
         <v>1.23</v>
@@ -1083,7 +1083,7 @@
         <v>46</v>
       </c>
       <c r="F19" s="6">
-        <v>1400</v>
+        <v>1520</v>
       </c>
       <c r="G19" s="3">
         <v>1.23</v>
@@ -1109,7 +1109,7 @@
         <v>46</v>
       </c>
       <c r="F20" s="6">
-        <v>8000</v>
+        <v>8140</v>
       </c>
       <c r="G20" s="3">
         <v>1.23</v>
@@ -1135,7 +1135,7 @@
         <v>46</v>
       </c>
       <c r="F21" s="6">
-        <v>10600</v>
+        <v>10917</v>
       </c>
       <c r="G21" s="3">
         <v>1.23</v>
@@ -1161,7 +1161,7 @@
         <v>46</v>
       </c>
       <c r="F22" s="6">
-        <v>6800</v>
+        <v>6875</v>
       </c>
       <c r="G22" s="3">
         <v>1.23</v>
@@ -1187,7 +1187,7 @@
         <v>46</v>
       </c>
       <c r="F23" s="6">
-        <v>1200</v>
+        <v>1260</v>
       </c>
       <c r="G23" s="3">
         <v>1.23</v>
@@ -1213,7 +1213,7 @@
         <v>46</v>
       </c>
       <c r="F24" s="6">
-        <v>3400</v>
+        <v>3356</v>
       </c>
       <c r="G24" s="3">
         <v>1.23</v>
@@ -1265,7 +1265,7 @@
         <v>46</v>
       </c>
       <c r="F26" s="6">
-        <v>2400</v>
+        <v>2377</v>
       </c>
       <c r="G26" s="3">
         <v>1.23</v>
@@ -1291,7 +1291,7 @@
         <v>46</v>
       </c>
       <c r="F27" s="6">
-        <v>7000</v>
+        <v>7098</v>
       </c>
       <c r="G27" s="3">
         <v>1.23</v>
@@ -1499,7 +1499,7 @@
         <v>46</v>
       </c>
       <c r="F35" s="6">
-        <v>17400</v>
+        <v>17901</v>
       </c>
       <c r="G35" s="3">
         <v>1.75</v>
@@ -1525,7 +1525,7 @@
         <v>46</v>
       </c>
       <c r="F36" s="6">
-        <v>1400</v>
+        <v>1510</v>
       </c>
       <c r="G36" s="3">
         <v>1.75</v>
@@ -1551,7 +1551,7 @@
         <v>46</v>
       </c>
       <c r="F37" s="6">
-        <v>8200</v>
+        <v>8172</v>
       </c>
       <c r="G37" s="3">
         <v>1.75</v>
@@ -1577,7 +1577,7 @@
         <v>46</v>
       </c>
       <c r="F38" s="6">
-        <v>800</v>
+        <v>2250</v>
       </c>
       <c r="G38" s="3">
         <v>1.75</v>
@@ -1603,7 +1603,7 @@
         <v>46</v>
       </c>
       <c r="F39" s="6">
-        <v>12600</v>
+        <v>13438</v>
       </c>
       <c r="G39" s="3">
         <v>1.75</v>
@@ -1629,7 +1629,7 @@
         <v>46</v>
       </c>
       <c r="F40" s="6">
-        <v>6800</v>
+        <v>8038</v>
       </c>
       <c r="G40" s="3">
         <v>1.75</v>
@@ -1655,7 +1655,7 @@
         <v>46</v>
       </c>
       <c r="F41" s="6">
-        <v>5000</v>
+        <v>5434</v>
       </c>
       <c r="G41" s="3">
         <v>1.75</v>
@@ -1681,7 +1681,7 @@
         <v>46</v>
       </c>
       <c r="F42" s="6">
-        <v>3600</v>
+        <v>3785</v>
       </c>
       <c r="G42" s="3">
         <v>1.75</v>
@@ -1863,7 +1863,7 @@
         <v>46</v>
       </c>
       <c r="F49" s="6">
-        <v>9811</v>
+        <v>10111</v>
       </c>
       <c r="G49" s="3">
         <v>1.75</v>
@@ -1889,7 +1889,7 @@
         <v>46</v>
       </c>
       <c r="F50" s="6">
-        <v>10000</v>
+        <v>10128</v>
       </c>
       <c r="G50" s="3">
         <v>1.75</v>
@@ -1915,7 +1915,7 @@
         <v>46</v>
       </c>
       <c r="F51" s="6">
-        <v>10000</v>
+        <v>10103</v>
       </c>
       <c r="G51" s="3">
         <v>1.75</v>

</xml_diff>